<commit_message>
Generate Self Onboarding and TeamHR backend workbooks
</commit_message>
<xml_diff>
--- a/data/masters/Self_Onboarding_Template.xlsx
+++ b/data/masters/Self_Onboarding_Template.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Onboarding" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Self Onboarding Upload" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Lists" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
@@ -18,17 +18,13 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="3">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <b val="1"/>
-      <color rgb="00FFFFFF"/>
     </font>
     <font>
       <b val="1"/>
@@ -43,11 +39,11 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="001F4E79"/>
+        <fgColor rgb="00D9E1F2"/>
       </patternFill>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -55,16 +51,21 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -430,88 +431,128 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K1"/>
+  <dimension ref="A1:N1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="6" customWidth="1" min="1" max="1"/>
+    <col width="24" customWidth="1" min="2" max="2"/>
+    <col width="15" customWidth="1" min="3" max="3"/>
+    <col width="24" customWidth="1" min="4" max="4"/>
+    <col width="10" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="16" customWidth="1" min="7" max="7"/>
+    <col width="18" customWidth="1" min="8" max="8"/>
+    <col width="14" customWidth="1" min="9" max="9"/>
+    <col width="32" customWidth="1" min="10" max="10"/>
+    <col width="18" customWidth="1" min="11" max="11"/>
+    <col width="14" customWidth="1" min="12" max="12"/>
+    <col width="34" customWidth="1" min="13" max="13"/>
+    <col width="30" customWidth="1" min="14" max="14"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Name</t>
+          <t>Sl No</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>Mobile</t>
+          <t>Name*</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>Team</t>
+          <t>Mobile Number*</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>Cost Code</t>
+          <t>Team*</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>Role / Designation</t>
+          <t>Cost Code*</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>Migrant</t>
+          <t>Migrant Bonus*</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>Facility Type</t>
+          <t>Facility Type*</t>
         </is>
       </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
-          <t>LOB / Sub Type</t>
+          <t>Line of Business*</t>
         </is>
       </c>
       <c r="I1" s="1" t="inlineStr">
         <is>
-          <t>State</t>
+          <t>Sub Type*</t>
         </is>
       </c>
       <c r="J1" s="1" t="inlineStr">
         <is>
-          <t>Contractor</t>
+          <t>Role - Designation*</t>
         </is>
       </c>
       <c r="K1" s="1" t="inlineStr">
         <is>
-          <t>Facility / Location Code</t>
+          <t>Fixed Net Take Home*</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>State*</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>Facility*</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>Contractor*</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <dataValidations count="7">
-    <dataValidation sqref="F2:F10000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"Yes,No"</formula1>
+  <dataValidations count="10">
+    <dataValidation sqref="D2:D2000" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Invalid value" error="Please pick a value from the dropdown list." type="list">
+      <formula1>=Lists!$B$2:$B$3</formula1>
     </dataValidation>
-    <dataValidation sqref="G2:G10000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"Delivery Hub"</formula1>
+    <dataValidation sqref="E2:E2000" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Invalid value" error="Please pick a value from the dropdown list." type="list">
+      <formula1>=Lists!$A$2:$A$5</formula1>
     </dataValidation>
-    <dataValidation sqref="D2:D10000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>=Lists!$A$2:$A$100</formula1>
+    <dataValidation sqref="F2:F2000" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Invalid value" error="Please pick a value from the dropdown list." type="list">
+      <formula1>=Lists!$F$2:$F$3</formula1>
     </dataValidation>
-    <dataValidation sqref="E2:E10000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>=Lists!$B$2:$B$100</formula1>
+    <dataValidation sqref="G2:G2000" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Invalid value" error="Please pick a value from the dropdown list." type="list">
+      <formula1>=Lists!$C$2:$C$4</formula1>
     </dataValidation>
-    <dataValidation sqref="H2:H10000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"Ekart"</formula1>
+    <dataValidation sqref="H2:H2000" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Invalid value" error="Please pick a value from the dropdown list." type="list">
+      <formula1>=Lists!$G$2:$G$2</formula1>
     </dataValidation>
-    <dataValidation sqref="J2:J10000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"TEAM HR"</formula1>
+    <dataValidation sqref="I2:I2000" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Invalid value" error="Please pick a value from the dropdown list." type="list">
+      <formula1>=Lists!$G$2:$G$2</formula1>
     </dataValidation>
-    <dataValidation sqref="I2:I10000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"Karnataka"</formula1>
+    <dataValidation sqref="J2:J2000" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Invalid value" error="Please pick a value from the dropdown list." type="list">
+      <formula1>=Lists!$D$2:$D$8</formula1>
+    </dataValidation>
+    <dataValidation sqref="L2:L2000" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Invalid value" error="Please pick a value from the dropdown list." type="list">
+      <formula1>=Lists!$H$2:$H$2</formula1>
+    </dataValidation>
+    <dataValidation sqref="M2:M2000" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Invalid value" error="Please pick a value from the dropdown list." type="list">
+      <formula1>=Lists!$E$2:$E$47</formula1>
+    </dataValidation>
+    <dataValidation sqref="N2:N2000" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Invalid value" error="Please pick a value from the dropdown list." type="list">
+      <formula1>=Lists!$I$2:$I$2</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -524,23 +565,53 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C47"/>
+  <dimension ref="A1:I47"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="2" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>Cost Codes</t>
         </is>
       </c>
-      <c r="B1" s="2" t="inlineStr">
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Teams</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Facility Types</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
         <is>
           <t>Designations</t>
         </is>
       </c>
-      <c r="C1" s="2" t="inlineStr">
-        <is>
-          <t>Locations</t>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>Facilities</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>Migrant</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>LOB / Sub Type</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>States</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>Contractors</t>
         </is>
       </c>
     </row>
@@ -552,12 +623,42 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
+          <t>LAST MILE - OPERATIONS</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>DELIVERY_HUB</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
           <t>LM - Delivery Executive</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>NelamangalaHub_BLR_PL</t>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>Nelamangala-PL</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>EKART</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>KARNATAKA</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>TEAM HR GSA PRIVATE LIMITED</t>
         </is>
       </c>
     </row>
@@ -569,12 +670,27 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
+          <t>FIRST MILE - OPERATIONS</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>PICKUP_HUB</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
           <t>LM - Sorter</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>BanaswadiHub_BLR_PL</t>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Banaswadi-PL</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -584,14 +700,19 @@
           <t>8751</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr">
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Needs Review</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
         <is>
           <t>LM - Team Leader</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>YelahankaHub_BLR_PL</t>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Yelahanka-PL</t>
         </is>
       </c>
     </row>
@@ -601,323 +722,323 @@
           <t>8752</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr">
+      <c r="D5" t="inlineStr">
         <is>
           <t>LM - Prexo Delivery Executive</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>ElectronicCityHub_BLR_PL</t>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Electronic City-PL</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="B6" t="inlineStr">
+      <c r="D6" t="inlineStr">
         <is>
           <t>FM - Delivery Executive</t>
         </is>
       </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>KR_PuramHub_BLR_PL</t>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>KR Puram-PL</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="B7" t="inlineStr">
+      <c r="D7" t="inlineStr">
         <is>
           <t>FM - Sorter</t>
         </is>
       </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>WhitefieldHub_BLR_PL</t>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>Whitefield-PL</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="B8" t="inlineStr">
+      <c r="D8" t="inlineStr">
         <is>
           <t>FM - Team Leader</t>
         </is>
       </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>MarathahalliHub_BLR_PL</t>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>Marathahalli-PL</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>HebbalHub_BLR_PL</t>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>Hebbal-PL</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>HSR_Hub_BLR_PL</t>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>HSR-PL</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>BTM_Hub_BLR_PL</t>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>BTM-PL</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="C12" t="inlineStr">
-        <is>
-          <t>JayanagarHub_BLR_PL</t>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>Jayanagar-PL</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="C13" t="inlineStr">
-        <is>
-          <t>KoramangalaHub_BLR_PL</t>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>Koramangala-PL</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="C14" t="inlineStr">
-        <is>
-          <t>IndiranagarHub_BLR_PL</t>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>Indiranagar-PL</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="C15" t="inlineStr">
-        <is>
-          <t>JP_NagarHub_BLR_PL</t>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>JP Nagar-PL</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="C16" t="inlineStr">
-        <is>
-          <t>PeenyaHub_BLR_PL</t>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>Peenya-PL</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="C17" t="inlineStr">
-        <is>
-          <t>RajajinagarHub_BLR_PL</t>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>Rajajinagar-PL</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="C18" t="inlineStr">
-        <is>
-          <t>BasavanagudiHub_BLR_PL</t>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>Basavanagudi-PL</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="C19" t="inlineStr">
-        <is>
-          <t>VijayanagarHub_BLR_PL</t>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>Vijayanagar-PL</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="C20" t="inlineStr">
-        <is>
-          <t>KengeriHub_BLR_PL</t>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>Kengeri-PL</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="C21" t="inlineStr">
-        <is>
-          <t>BannerghattaHub_BLR_PL</t>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>Bannerghatta-PL</t>
         </is>
       </c>
     </row>
     <row r="22">
-      <c r="C22" t="inlineStr">
-        <is>
-          <t>NelamangalaHub_BLR</t>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>Nelamangala</t>
         </is>
       </c>
     </row>
     <row r="23">
-      <c r="C23" t="inlineStr">
-        <is>
-          <t>BanaswadiHub_BLR</t>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>Banaswadi</t>
         </is>
       </c>
     </row>
     <row r="24">
-      <c r="C24" t="inlineStr">
-        <is>
-          <t>YelahankaHub_BLR</t>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>Yelahanka</t>
         </is>
       </c>
     </row>
     <row r="25">
-      <c r="C25" t="inlineStr">
-        <is>
-          <t>ElectronicCityHub_BLR</t>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>Electronic City</t>
         </is>
       </c>
     </row>
     <row r="26">
-      <c r="C26" t="inlineStr">
-        <is>
-          <t>KR_PuramHub_BLR</t>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>KR Puram</t>
         </is>
       </c>
     </row>
     <row r="27">
-      <c r="C27" t="inlineStr">
-        <is>
-          <t>WhitefieldHub_BLR</t>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>Whitefield</t>
         </is>
       </c>
     </row>
     <row r="28">
-      <c r="C28" t="inlineStr">
-        <is>
-          <t>MarathahalliHub_BLR</t>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>Marathahalli</t>
         </is>
       </c>
     </row>
     <row r="29">
-      <c r="C29" t="inlineStr">
-        <is>
-          <t>HebbalHub_BLR</t>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>Hebbal</t>
         </is>
       </c>
     </row>
     <row r="30">
-      <c r="C30" t="inlineStr">
-        <is>
-          <t>HSR_Hub_BLR</t>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>HSR</t>
         </is>
       </c>
     </row>
     <row r="31">
-      <c r="C31" t="inlineStr">
-        <is>
-          <t>BTM_Hub_BLR</t>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>BTM</t>
         </is>
       </c>
     </row>
     <row r="32">
-      <c r="C32" t="inlineStr">
-        <is>
-          <t>JayanagarHub_BLR</t>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>Jayanagar</t>
         </is>
       </c>
     </row>
     <row r="33">
-      <c r="C33" t="inlineStr">
-        <is>
-          <t>KoramangalaHub_BLR</t>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>Koramangala</t>
         </is>
       </c>
     </row>
     <row r="34">
-      <c r="C34" t="inlineStr">
-        <is>
-          <t>IndiranagarHub_BLR</t>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>Indiranagar</t>
         </is>
       </c>
     </row>
     <row r="35">
-      <c r="C35" t="inlineStr">
-        <is>
-          <t>JP_NagarHub_BLR</t>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>JP Nagar</t>
         </is>
       </c>
     </row>
     <row r="36">
-      <c r="C36" t="inlineStr">
-        <is>
-          <t>PeenyaHub_BLR</t>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>Peenya</t>
         </is>
       </c>
     </row>
     <row r="37">
-      <c r="C37" t="inlineStr">
-        <is>
-          <t>RajajinagarHub_BLR</t>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>Rajajinagar</t>
         </is>
       </c>
     </row>
     <row r="38">
-      <c r="C38" t="inlineStr">
-        <is>
-          <t>BasavanagudiHub_BLR</t>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>Basavanagudi</t>
         </is>
       </c>
     </row>
     <row r="39">
-      <c r="C39" t="inlineStr">
-        <is>
-          <t>VijayanagarHub_BLR</t>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>Vijayanagar</t>
         </is>
       </c>
     </row>
     <row r="40">
-      <c r="C40" t="inlineStr">
-        <is>
-          <t>KengeriHub_BLR</t>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>Kengeri</t>
         </is>
       </c>
     </row>
     <row r="41">
-      <c r="C41" t="inlineStr">
-        <is>
-          <t>BannerghattaHub_BLR</t>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>Bannerghatta</t>
         </is>
       </c>
     </row>
     <row r="42">
-      <c r="C42" t="inlineStr">
-        <is>
-          <t>BanaswadiMYNTRAHub_BLR</t>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>BanaswadiMYNTRA</t>
         </is>
       </c>
     </row>
     <row r="43">
-      <c r="C43" t="inlineStr">
-        <is>
-          <t>HebbalMYNTRAHub_BLR</t>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>HebbalMYNTRA</t>
         </is>
       </c>
     </row>
     <row r="44">
-      <c r="C44" t="inlineStr">
-        <is>
-          <t>KoramangalaMYNTRAHub_BLR</t>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>KoramangalaMYNTRA</t>
         </is>
       </c>
     </row>
     <row r="45">
-      <c r="C45" t="inlineStr">
-        <is>
-          <t>HSR_MYNTRAHub_BLR</t>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>HSRMYNTRA</t>
         </is>
       </c>
     </row>
     <row r="46">
-      <c r="C46" t="inlineStr">
-        <is>
-          <t>WhitefieldMYNTRAHub_BLR</t>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>WhitefieldMYNTRA</t>
         </is>
       </c>
     </row>
     <row r="47">
-      <c r="C47" t="inlineStr">
-        <is>
-          <t>MarathahalliMYNTRAHub_BLR</t>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>MarathahalliMYNTRA</t>
         </is>
       </c>
     </row>

</xml_diff>